<commit_message>
Fix some issues in verify page in ui
</commit_message>
<xml_diff>
--- a/docs/samples/Special Projects Pillar'25 service letters.xlsx
+++ b/docs/samples/Special Projects Pillar'25 service letters.xlsx
@@ -1,17 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20417"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DN-75\Edu\DN\Mora Spirit\pdf_generator\docs\samples\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{576BF9A5-69E6-4F89-B816-5715BEAB3CC1}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="8424" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet state="visible" name="Sheet1" sheetId="1" r:id="rId5"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="214" uniqueCount="101">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="256" uniqueCount="105">
   <si>
     <t>Member ID</t>
   </si>
@@ -325,30 +334,44 @@
   </si>
   <si>
     <t>Yasiru Chandula</t>
+  </si>
+  <si>
+    <t>Pillar</t>
+  </si>
+  <si>
+    <t>Start Date</t>
+  </si>
+  <si>
+    <t>End Date</t>
+  </si>
+  <si>
+    <t>Web</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="4">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
-      <sz val="10.0"/>
+      <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
     </font>
     <font>
-      <sz val="11.0"/>
+      <sz val="11"/>
       <color theme="1"/>
       <name val="Arial"/>
       <scheme val="minor"/>
@@ -359,7 +382,7 @@
       <patternFill patternType="none"/>
     </fill>
     <fill>
-      <patternFill patternType="lightGray"/>
+      <patternFill patternType="gray125"/>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -368,8 +391,14 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
-    <border/>
+  <borders count="4">
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
     <border>
       <left style="thin">
         <color rgb="FF000000"/>
@@ -383,43 +412,61 @@
       <bottom style="thin">
         <color rgb="FF000000"/>
       </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="1" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="1" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf borderId="1" fillId="2" fontId="1" numFmtId="0" xfId="0" applyBorder="1" applyFill="1" applyFont="1"/>
-    <xf borderId="1" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="2" fontId="1" numFmtId="0" xfId="0" applyFill="1" applyFont="1"/>
+  <cellXfs count="13">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle xfId="0" name="Normal" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
 </file>
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
@@ -427,7 +474,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheets">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Sheets">
   <a:themeElements>
     <a:clrScheme name="Sheets">
       <a:dk1>
@@ -617,23 +664,27 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <dimension ref="A1:Z40"/>
+  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col customWidth="1" min="2" max="2" width="20.13"/>
-    <col customWidth="1" min="4" max="4" width="13.75"/>
-    <col customWidth="1" min="5" max="5" width="140.38"/>
-    <col customWidth="1" min="6" max="6" width="178.13"/>
+    <col min="2" max="2" width="20.109375" customWidth="1"/>
+    <col min="4" max="4" width="13.77734375" customWidth="1"/>
+    <col min="5" max="5" width="187.77734375" customWidth="1"/>
+    <col min="6" max="6" width="255.44140625" customWidth="1"/>
+    <col min="9" max="9" width="12.6640625" style="10"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -652,8 +703,17 @@
       <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="2">
+      <c r="G1" s="9" t="s">
+        <v>101</v>
+      </c>
+      <c r="H1" s="9" t="s">
+        <v>102</v>
+      </c>
+      <c r="I1" s="11" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="2" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>6</v>
       </c>
@@ -670,8 +730,17 @@
         <v>10</v>
       </c>
       <c r="F2" s="3"/>
-    </row>
-    <row r="3">
+      <c r="G2" s="9" t="s">
+        <v>104</v>
+      </c>
+      <c r="H2" s="10">
+        <v>45275</v>
+      </c>
+      <c r="I2" s="12">
+        <v>45961</v>
+      </c>
+    </row>
+    <row r="3" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>11</v>
       </c>
@@ -690,8 +759,17 @@
       <c r="F3" s="1" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="4">
+      <c r="G3" s="9" t="s">
+        <v>104</v>
+      </c>
+      <c r="H3" s="10">
+        <v>45276</v>
+      </c>
+      <c r="I3" s="12">
+        <v>45962</v>
+      </c>
+    </row>
+    <row r="4" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>16</v>
       </c>
@@ -708,8 +786,17 @@
         <v>10</v>
       </c>
       <c r="F4" s="3"/>
-    </row>
-    <row r="5">
+      <c r="G4" s="9" t="s">
+        <v>104</v>
+      </c>
+      <c r="H4" s="10">
+        <v>45277</v>
+      </c>
+      <c r="I4" s="12">
+        <v>45963</v>
+      </c>
+    </row>
+    <row r="5" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>18</v>
       </c>
@@ -728,8 +815,17 @@
       <c r="F5" s="4" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="6">
+      <c r="G5" s="9" t="s">
+        <v>104</v>
+      </c>
+      <c r="H5" s="10">
+        <v>45278</v>
+      </c>
+      <c r="I5" s="12">
+        <v>45964</v>
+      </c>
+    </row>
+    <row r="6" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>21</v>
       </c>
@@ -745,8 +841,17 @@
       <c r="E6" s="1" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="7">
+      <c r="G6" s="9" t="s">
+        <v>104</v>
+      </c>
+      <c r="H6" s="10">
+        <v>45279</v>
+      </c>
+      <c r="I6" s="12">
+        <v>45965</v>
+      </c>
+    </row>
+    <row r="7" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>23</v>
       </c>
@@ -763,8 +868,17 @@
         <v>10</v>
       </c>
       <c r="F7" s="3"/>
-    </row>
-    <row r="8">
+      <c r="G7" s="9" t="s">
+        <v>104</v>
+      </c>
+      <c r="H7" s="10">
+        <v>45280</v>
+      </c>
+      <c r="I7" s="12">
+        <v>45966</v>
+      </c>
+    </row>
+    <row r="8" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>25</v>
       </c>
@@ -781,8 +895,17 @@
         <v>10</v>
       </c>
       <c r="F8" s="3"/>
-    </row>
-    <row r="9">
+      <c r="G8" s="9" t="s">
+        <v>104</v>
+      </c>
+      <c r="H8" s="10">
+        <v>45281</v>
+      </c>
+      <c r="I8" s="12">
+        <v>45967</v>
+      </c>
+    </row>
+    <row r="9" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>27</v>
       </c>
@@ -801,8 +924,17 @@
       <c r="F9" s="4" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="10">
+      <c r="G9" s="9" t="s">
+        <v>104</v>
+      </c>
+      <c r="H9" s="10">
+        <v>45282</v>
+      </c>
+      <c r="I9" s="12">
+        <v>45968</v>
+      </c>
+    </row>
+    <row r="10" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>30</v>
       </c>
@@ -821,8 +953,17 @@
       <c r="F10" s="4" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="11">
+      <c r="G10" s="9" t="s">
+        <v>104</v>
+      </c>
+      <c r="H10" s="10">
+        <v>45283</v>
+      </c>
+      <c r="I10" s="12">
+        <v>45969</v>
+      </c>
+    </row>
+    <row r="11" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
         <v>33</v>
       </c>
@@ -833,9 +974,15 @@
       <c r="D11" s="6"/>
       <c r="E11" s="7"/>
       <c r="F11" s="6"/>
-      <c r="G11" s="8"/>
-      <c r="H11" s="8"/>
-      <c r="I11" s="8"/>
+      <c r="G11" s="9" t="s">
+        <v>104</v>
+      </c>
+      <c r="H11" s="10">
+        <v>45284</v>
+      </c>
+      <c r="I11" s="12">
+        <v>45970</v>
+      </c>
       <c r="J11" s="8"/>
       <c r="K11" s="8"/>
       <c r="L11" s="8"/>
@@ -854,7 +1001,7 @@
       <c r="Y11" s="8"/>
       <c r="Z11" s="8"/>
     </row>
-    <row r="12">
+    <row r="12" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>35</v>
       </c>
@@ -871,8 +1018,17 @@
         <v>10</v>
       </c>
       <c r="F12" s="3"/>
-    </row>
-    <row r="13">
+      <c r="G12" s="9" t="s">
+        <v>104</v>
+      </c>
+      <c r="H12" s="10">
+        <v>45285</v>
+      </c>
+      <c r="I12" s="12">
+        <v>45971</v>
+      </c>
+    </row>
+    <row r="13" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>37</v>
       </c>
@@ -891,8 +1047,17 @@
       <c r="F13" s="4" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="14">
+      <c r="G13" s="9" t="s">
+        <v>104</v>
+      </c>
+      <c r="H13" s="10">
+        <v>45286</v>
+      </c>
+      <c r="I13" s="12">
+        <v>45972</v>
+      </c>
+    </row>
+    <row r="14" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>40</v>
       </c>
@@ -911,8 +1076,17 @@
       <c r="F14" s="4" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="15">
+      <c r="G14" s="9" t="s">
+        <v>104</v>
+      </c>
+      <c r="H14" s="10">
+        <v>45287</v>
+      </c>
+      <c r="I14" s="12">
+        <v>45973</v>
+      </c>
+    </row>
+    <row r="15" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>43</v>
       </c>
@@ -929,8 +1103,17 @@
         <v>10</v>
       </c>
       <c r="F15" s="3"/>
-    </row>
-    <row r="16">
+      <c r="G15" s="9" t="s">
+        <v>104</v>
+      </c>
+      <c r="H15" s="10">
+        <v>45288</v>
+      </c>
+      <c r="I15" s="12">
+        <v>45974</v>
+      </c>
+    </row>
+    <row r="16" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>45</v>
       </c>
@@ -949,8 +1132,17 @@
       <c r="F16" s="4" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="17">
+      <c r="G16" s="9" t="s">
+        <v>104</v>
+      </c>
+      <c r="H16" s="10">
+        <v>45289</v>
+      </c>
+      <c r="I16" s="12">
+        <v>45975</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>48</v>
       </c>
@@ -967,8 +1159,17 @@
         <v>10</v>
       </c>
       <c r="F17" s="3"/>
-    </row>
-    <row r="18">
+      <c r="G17" s="9" t="s">
+        <v>104</v>
+      </c>
+      <c r="H17" s="10">
+        <v>45290</v>
+      </c>
+      <c r="I17" s="12">
+        <v>45976</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
         <v>50</v>
       </c>
@@ -985,8 +1186,17 @@
         <v>10</v>
       </c>
       <c r="F18" s="3"/>
-    </row>
-    <row r="19">
+      <c r="G18" s="9" t="s">
+        <v>104</v>
+      </c>
+      <c r="H18" s="10">
+        <v>45291</v>
+      </c>
+      <c r="I18" s="12">
+        <v>45977</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
         <v>52</v>
       </c>
@@ -1003,8 +1213,17 @@
         <v>10</v>
       </c>
       <c r="F19" s="3"/>
-    </row>
-    <row r="20">
+      <c r="G19" s="9" t="s">
+        <v>104</v>
+      </c>
+      <c r="H19" s="10">
+        <v>45292</v>
+      </c>
+      <c r="I19" s="12">
+        <v>45978</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
         <v>54</v>
       </c>
@@ -1023,8 +1242,17 @@
       <c r="F20" s="4" t="s">
         <v>56</v>
       </c>
-    </row>
-    <row r="21">
+      <c r="G20" s="9" t="s">
+        <v>104</v>
+      </c>
+      <c r="H20" s="10">
+        <v>45293</v>
+      </c>
+      <c r="I20" s="12">
+        <v>45979</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
         <v>57</v>
       </c>
@@ -1043,8 +1271,17 @@
       <c r="F21" s="4" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="22">
+      <c r="G21" s="9" t="s">
+        <v>104</v>
+      </c>
+      <c r="H21" s="10">
+        <v>45294</v>
+      </c>
+      <c r="I21" s="12">
+        <v>45980</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
         <v>60</v>
       </c>
@@ -1063,8 +1300,17 @@
       <c r="F22" s="4" t="s">
         <v>62</v>
       </c>
-    </row>
-    <row r="23">
+      <c r="G22" s="9" t="s">
+        <v>104</v>
+      </c>
+      <c r="H22" s="10">
+        <v>45295</v>
+      </c>
+      <c r="I22" s="12">
+        <v>45981</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
         <v>63</v>
       </c>
@@ -1081,8 +1327,17 @@
         <v>10</v>
       </c>
       <c r="F23" s="3"/>
-    </row>
-    <row r="24">
+      <c r="G23" s="9" t="s">
+        <v>104</v>
+      </c>
+      <c r="H23" s="10">
+        <v>45296</v>
+      </c>
+      <c r="I23" s="12">
+        <v>45982</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
         <v>65</v>
       </c>
@@ -1101,8 +1356,17 @@
       <c r="F24" s="1" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="25">
+      <c r="G24" s="9" t="s">
+        <v>104</v>
+      </c>
+      <c r="H24" s="10">
+        <v>45297</v>
+      </c>
+      <c r="I24" s="12">
+        <v>45983</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
         <v>67</v>
       </c>
@@ -1119,8 +1383,17 @@
         <v>10</v>
       </c>
       <c r="F25" s="3"/>
-    </row>
-    <row r="26">
+      <c r="G25" s="9" t="s">
+        <v>104</v>
+      </c>
+      <c r="H25" s="10">
+        <v>45298</v>
+      </c>
+      <c r="I25" s="12">
+        <v>45984</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
         <v>69</v>
       </c>
@@ -1137,8 +1410,17 @@
         <v>10</v>
       </c>
       <c r="F26" s="3"/>
-    </row>
-    <row r="27">
+      <c r="G26" s="9" t="s">
+        <v>104</v>
+      </c>
+      <c r="H26" s="10">
+        <v>45299</v>
+      </c>
+      <c r="I26" s="12">
+        <v>45985</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
         <v>71</v>
       </c>
@@ -1157,8 +1439,17 @@
       <c r="F27" s="4" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="28">
+      <c r="G27" s="9" t="s">
+        <v>104</v>
+      </c>
+      <c r="H27" s="10">
+        <v>45300</v>
+      </c>
+      <c r="I27" s="12">
+        <v>45986</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
         <v>74</v>
       </c>
@@ -1177,8 +1468,17 @@
       <c r="F28" s="4" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="29">
+      <c r="G28" s="9" t="s">
+        <v>104</v>
+      </c>
+      <c r="H28" s="10">
+        <v>45301</v>
+      </c>
+      <c r="I28" s="12">
+        <v>45987</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
         <v>76</v>
       </c>
@@ -1195,8 +1495,17 @@
         <v>10</v>
       </c>
       <c r="F29" s="3"/>
-    </row>
-    <row r="30">
+      <c r="G29" s="9" t="s">
+        <v>104</v>
+      </c>
+      <c r="H29" s="10">
+        <v>45302</v>
+      </c>
+      <c r="I29" s="12">
+        <v>45988</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
         <v>78</v>
       </c>
@@ -1213,8 +1522,17 @@
         <v>10</v>
       </c>
       <c r="F30" s="3"/>
-    </row>
-    <row r="31">
+      <c r="G30" s="9" t="s">
+        <v>104</v>
+      </c>
+      <c r="H30" s="10">
+        <v>45303</v>
+      </c>
+      <c r="I30" s="12">
+        <v>45989</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
         <v>80</v>
       </c>
@@ -1231,8 +1549,17 @@
         <v>10</v>
       </c>
       <c r="F31" s="3"/>
-    </row>
-    <row r="32">
+      <c r="G31" s="9" t="s">
+        <v>104</v>
+      </c>
+      <c r="H31" s="10">
+        <v>45304</v>
+      </c>
+      <c r="I31" s="12">
+        <v>45990</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
         <v>82</v>
       </c>
@@ -1249,8 +1576,17 @@
         <v>10</v>
       </c>
       <c r="F32" s="3"/>
-    </row>
-    <row r="33">
+      <c r="G32" s="9" t="s">
+        <v>104</v>
+      </c>
+      <c r="H32" s="10">
+        <v>45305</v>
+      </c>
+      <c r="I32" s="12">
+        <v>45991</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
         <v>84</v>
       </c>
@@ -1269,8 +1605,17 @@
       <c r="F33" s="1" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="34">
+      <c r="G33" s="9" t="s">
+        <v>104</v>
+      </c>
+      <c r="H33" s="10">
+        <v>45306</v>
+      </c>
+      <c r="I33" s="12">
+        <v>45992</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
         <v>86</v>
       </c>
@@ -1287,8 +1632,17 @@
         <v>10</v>
       </c>
       <c r="F34" s="3"/>
-    </row>
-    <row r="35">
+      <c r="G34" s="9" t="s">
+        <v>104</v>
+      </c>
+      <c r="H34" s="10">
+        <v>45307</v>
+      </c>
+      <c r="I34" s="12">
+        <v>45993</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
         <v>88</v>
       </c>
@@ -1307,8 +1661,17 @@
       <c r="F35" s="4" t="s">
         <v>90</v>
       </c>
-    </row>
-    <row r="36">
+      <c r="G35" s="9" t="s">
+        <v>104</v>
+      </c>
+      <c r="H35" s="10">
+        <v>45308</v>
+      </c>
+      <c r="I35" s="12">
+        <v>45994</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
         <v>91</v>
       </c>
@@ -1325,8 +1688,17 @@
         <v>10</v>
       </c>
       <c r="F36" s="3"/>
-    </row>
-    <row r="37">
+      <c r="G36" s="9" t="s">
+        <v>104</v>
+      </c>
+      <c r="H36" s="10">
+        <v>45309</v>
+      </c>
+      <c r="I36" s="12">
+        <v>45995</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
         <v>93</v>
       </c>
@@ -1343,8 +1715,17 @@
         <v>10</v>
       </c>
       <c r="F37" s="3"/>
-    </row>
-    <row r="38">
+      <c r="G37" s="9" t="s">
+        <v>104</v>
+      </c>
+      <c r="H37" s="10">
+        <v>45310</v>
+      </c>
+      <c r="I37" s="12">
+        <v>45996</v>
+      </c>
+    </row>
+    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
         <v>95</v>
       </c>
@@ -1361,8 +1742,17 @@
         <v>10</v>
       </c>
       <c r="F38" s="3"/>
-    </row>
-    <row r="39">
+      <c r="G38" s="9" t="s">
+        <v>104</v>
+      </c>
+      <c r="H38" s="10">
+        <v>45311</v>
+      </c>
+      <c r="I38" s="12">
+        <v>45997</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
         <v>97</v>
       </c>
@@ -1381,8 +1771,17 @@
       <c r="F39" s="1" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="40">
+      <c r="G39" s="9" t="s">
+        <v>104</v>
+      </c>
+      <c r="H39" s="10">
+        <v>45312</v>
+      </c>
+      <c r="I39" s="12">
+        <v>45998</v>
+      </c>
+    </row>
+    <row r="40" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
         <v>99</v>
       </c>
@@ -1399,16 +1798,26 @@
         <v>10</v>
       </c>
       <c r="F40" s="3"/>
+      <c r="G40" s="9" t="s">
+        <v>104</v>
+      </c>
+      <c r="H40" s="10">
+        <v>45313</v>
+      </c>
+      <c r="I40" s="12">
+        <v>45999</v>
+      </c>
     </row>
   </sheetData>
-  <dataValidations>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D1:D40">
+  <dataValidations count="2">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D1:D40" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"Letter type,General,Special"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="C1:C40">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="C1:C40" xr:uid="{00000000-0002-0000-0000-000001000000}">
       <formula1>"Gender,Male,Female"</formula1>
     </dataValidation>
   </dataValidations>
-  <drawing r:id="rId1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>